<commit_message>
Added Assertions and Extent Report
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/44b07c9c05f0c50c/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Udemy_CG_Sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{045ED0F3-F548-48E1-8D81-B3B248DDC972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6288E025-EABC-43CE-968D-BE33D80FCCC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="2148" windowWidth="17280" windowHeight="8880" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="CourseData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>TC_ID</t>
   </si>
@@ -70,6 +71,39 @@
   </si>
   <si>
     <t>zzzz111</t>
+  </si>
+  <si>
+    <t>Sap</t>
+  </si>
+  <si>
+    <t>C# Automation</t>
+  </si>
+  <si>
+    <t>Course Name</t>
+  </si>
+  <si>
+    <t>T_001</t>
+  </si>
+  <si>
+    <t>Selenium Webdriver</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>asdfghikl123</t>
+  </si>
+  <si>
+    <t>TC_006</t>
   </si>
 </sst>
 </file>
@@ -113,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,6 +155,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,14 +471,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14298DB-FA52-443D-8EE0-0C2038A39564}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -454,7 +489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -465,7 +500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -476,7 +511,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -485,6 +520,76 @@
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A14B4B03-4F81-4285-9453-B01353F6BA8A}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mylearing: improved AllCourses flow, integrated Excel utility, fixed cookie-based login issues and removed signup dependency
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/44b07c9c05f0c50c/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preet\Documents\Udemy_CG_Sprint\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{045ED0F3-F548-48E1-8D81-B3B248DDC972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98CEB51-A5D5-436F-9C49-9D0AF98E4C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="2148" windowWidth="17280" windowHeight="8880" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Courses" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -490,4 +491,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533DD918-D856-4D7C-A578-FDF45ECEB08B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
explore: added all the files
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/44b07c9c05f0c50c/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{045ED0F3-F548-48E1-8D81-B3B248DDC972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{8748306D-1E4A-455B-ADCC-204C45C278F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="2148" windowWidth="17280" windowHeight="8880" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>TC_ID</t>
   </si>
@@ -70,13 +66,19 @@
   </si>
   <si>
     <t>zzzz111</t>
+  </si>
+  <si>
+    <t>Email_id</t>
+  </si>
+  <si>
+    <t>kiruthikaa.nrs@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,6 +90,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -110,10 +120,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,8 +132,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -435,15 +451,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14298DB-FA52-443D-8EE0-0C2038A39564}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.21875" customWidth="1"/>
     <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="4" max="4" width="27.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -453,8 +470,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -464,8 +484,11 @@
       <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -476,7 +499,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -488,6 +511,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{490AC322-DFC4-4DB8-94E1-DC65D7D01C8F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
search-management: restored overwritten tesdata.xlsx
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,36 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{8748306D-1E4A-455B-ADCC-204C45C278F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Udemy_CG_Sprint\src\test\resources\testdata\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A45A7FF6-2153-4575-A602-3BDD94DA3B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="CourseData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>TC_ID</t>
   </si>
@@ -72,13 +68,46 @@
   </si>
   <si>
     <t>kiruthikaa.nrs@gmail.com</t>
+  </si>
+  <si>
+    <t>TC_001</t>
+  </si>
+  <si>
+    <t>Course Name</t>
+  </si>
+  <si>
+    <t>Selenium Webdriver</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>Sap</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>asdifg1234</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>C# Automation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,6 +127,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -124,7 +159,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,6 +171,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -452,15 +488,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14298DB-FA52-443D-8EE0-0C2038A39564}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -474,7 +510,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -488,7 +524,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -499,7 +535,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -516,4 +552,74 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F8109AB-4BF8-402D-8BBB-BA3F1EA1CE26}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
my-learning: completed all features with scenario outline and parallel execution
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -3,22 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Udemy_CG_Sprint\src\test\resources\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C910F162-E102-4FA7-9920-DE9A1B459558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{9C9DEEA9-FC97-4ACA-8CB2-941C96250B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C365673B-65E1-467A-9C19-10EFE90A9B55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Courses" sheetId="2" r:id="rId2"/>
-    <sheet name="CourseData" sheetId="3" r:id="rId3"/>
-    <sheet name="Explore" sheetId="4" r:id="rId4"/>
+    <sheet name="CourseData" sheetId="3" r:id="rId2"/>
+    <sheet name="Explore" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:P22"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
     <t>TC_ID</t>
   </si>
@@ -112,13 +107,25 @@
   </si>
   <si>
     <t>kiruthikaa.nrs@gmail.com</t>
+  </si>
+  <si>
+    <t>Cucumber</t>
+  </si>
+  <si>
+    <t>TestNG</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>TC_008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +149,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -164,7 +183,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -174,6 +193,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -490,14 +513,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14298DB-FA52-443D-8EE0-0C2038A39564}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -508,7 +531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -519,7 +542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -530,7 +553,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -547,97 +570,105 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533DD918-D856-4D7C-A578-FDF45ECEB08B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5632812A-6796-4DA8-8BC4-7CDE6C9763C7}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5632812A-6796-4DA8-8BC4-7CDE6C9763C7}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA44D535-C03C-4ABA-B01D-E481CBBAF896}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA44D535-C03C-4ABA-B01D-E481CBBAF896}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>

</xml_diff>